<commit_message>
feat(*): release csvx demo
</commit_message>
<xml_diff>
--- a/examples/chinese-sales.xlsx
+++ b/examples/chinese-sales.xlsx
@@ -398,7 +398,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:H4"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -420,7 +420,10 @@
         <v>含税销售额</v>
       </c>
       <c r="G1" t="str">
-        <v>平均数量</v>
+        <v>累计销售额</v>
+      </c>
+      <c r="H1" t="str">
+        <v>前一销售额</v>
       </c>
     </row>
     <row r="2">
@@ -440,10 +443,10 @@
         <v>15</v>
       </c>
       <c r="F2">
-        <v>16.2</v>
+        <v>15.39</v>
       </c>
       <c r="G2">
-        <v>6.333333333333333</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
@@ -463,10 +466,13 @@
         <v>16</v>
       </c>
       <c r="F3">
-        <v>17.28</v>
+        <v>16.42</v>
       </c>
       <c r="G3">
-        <v>6.333333333333333</v>
+        <v>31</v>
+      </c>
+      <c r="H3">
+        <v>15</v>
       </c>
     </row>
     <row r="4">
@@ -486,15 +492,18 @@
         <v>24</v>
       </c>
       <c r="F4">
-        <v>25.92</v>
+        <v>24.62</v>
       </c>
       <c r="G4">
-        <v>6.333333333333333</v>
+        <v>55</v>
+      </c>
+      <c r="H4">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H4"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -537,22 +546,22 @@
         <v>销售表</v>
       </c>
       <c r="C2" t="str">
-        <v>销售额与含税销售额</v>
+        <v>销售额与累计销售额</v>
       </c>
       <c r="D2" t="str">
         <v>销售额</v>
       </c>
       <c r="E2" t="str">
-        <v>含税销售额</v>
+        <v>累计销售额</v>
       </c>
       <c r="F2" t="str">
         <v/>
       </c>
       <c r="G2" t="str">
-        <v>销售额,含税销售额</v>
+        <v>销售额,累计销售额</v>
       </c>
       <c r="H2" t="str">
-        <v>{"$schema":"https://vega.github.io/schema/vega-lite/v5.json","mark":"bar","title":"销售额与含税销售额","data":{"values":[{"销售额":15,"含税销售额":16.2},{"销售额":16,"含税销售额":17.28},{"销售额":24,"含税销售额":25.92}]},"encoding":{"x":{"field":"销售额","type":"quantitative"},"y":{"field":"含税销售额","type":"quantitative"}}}</v>
+        <v>{"$schema":"https://vega.github.io/schema/vega-lite/v5.json","mark":"bar","title":"销售额与累计销售额","data":{"values":[{"销售额":15,"累计销售额":15},{"销售额":16,"累计销售额":31},{"销售额":24,"累计销售额":55}]},"encoding":{"x":{"field":"销售额","type":"quantitative"},"y":{"field":"累计销售额","type":"quantitative"}}}</v>
       </c>
     </row>
   </sheetData>

</xml_diff>